<commit_message>
Add GUI-based packing list workflow and update generated Excel outputs.
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="7000"/>
+    <workbookView windowWidth="18600" windowHeight="7000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="8">
-        <v>74700910</v>
+        <v>17000060</v>
       </c>
       <c r="D3" s="7">
         <v>1</v>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="8">
-        <v>17003230</v>
+        <v>17000240</v>
       </c>
       <c r="D9" s="17">
         <v>1</v>

</xml_diff>

<commit_message>
Update app, templates, and output workbooks
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="18600" windowHeight="7000"/>
+    <workbookView windowWidth="19200" windowHeight="7000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="75">
   <si>
     <t>序号</t>
   </si>
@@ -94,22 +94,7 @@
     <t>净重</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>ODBC</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>定制线</t>
-    </r>
+    <t>ODBC定制线</t>
   </si>
   <si>
     <t>DRW-WR-ODBC-V@10CA5&amp;S71</t>
@@ -127,30 +112,7 @@
     <t>220*150*120mm</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>IRME-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>垫片</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>-ODBC</t>
-    </r>
+    <t>IRME-垫片-ODBC</t>
   </si>
   <si>
     <t>DRW-Part-ODBC-0260</t>
@@ -168,88 +130,19 @@
     <t>M4X10 ，不锈钢</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>Maintenance</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>标签</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>-ODBC</t>
-    </r>
+    <t>Maintenance标签-ODBC</t>
   </si>
   <si>
     <t>DRW-Pst-ODBC-8032</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>ERME-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>吸头套筒</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>-ODBC</t>
-    </r>
+    <t>ERME-吸头套筒-ODBC</t>
   </si>
   <si>
     <t>DRW-Part-ODBC-0344</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>SLIN-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>垫硅胶</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>-ODBC</t>
-    </r>
+    <t>SLIN-垫硅胶-ODBC</t>
   </si>
   <si>
     <t>DRW-Part-ODBC-0311</t>
@@ -261,88 +154,19 @@
     <t>DRW-Part-ODBC-0323</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>SLIN-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>静电计支撑板</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>-ODBC</t>
-    </r>
+    <t>SLIN-静电计支撑板-ODBC</t>
   </si>
   <si>
     <t>DRW-Part-ODBC-0332</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>SLIN-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>静电计固定板</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>-ODBC</t>
-    </r>
+    <t>SLIN-静电计固定板-ODBC</t>
   </si>
   <si>
     <t>DRW-Part-ODBC-0333</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>SLIN-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="微软雅黑"/>
-        <charset val="134"/>
-      </rPr>
-      <t>硅胶防撞堵头</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>-ODBC</t>
-    </r>
+    <t>SLIN-硅胶防撞堵头-ODBC</t>
   </si>
   <si>
     <t>DRW-Part-ODBC-0310</t>
@@ -361,9 +185,6 @@
   </si>
   <si>
     <t>D</t>
-  </si>
-  <si>
-    <t>ODBC定制线</t>
   </si>
   <si>
     <t>DRW-WR-ODBC-VA46EA1</t>
@@ -451,7 +272,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -467,14 +288,21 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="major"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -492,14 +320,23 @@
     </font>
     <font>
       <sz val="11"/>
-      <name val="微软雅黑"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="ARIAL"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="major"/>
     </font>
     <font>
       <u/>
@@ -844,7 +681,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -885,19 +722,6 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -1024,137 +848,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1178,57 +1002,63 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="6" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1635,28 +1465,28 @@
         <v>1</v>
       </c>
       <c r="E2" s="9"/>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="12" t="s">
+      <c r="H2" s="12"/>
+      <c r="I2" s="12"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="12"/>
+      <c r="Q2" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="R2" s="11" t="s">
+      <c r="R2" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="S2" s="11"/>
+      <c r="S2" s="12"/>
     </row>
     <row r="3" s="1" customFormat="1" ht="13" customHeight="1" spans="1:19">
       <c r="A3" s="7">
@@ -1669,29 +1499,29 @@
       <c r="D3" s="7">
         <v>1</v>
       </c>
-      <c r="E3" s="13"/>
-      <c r="F3" s="8" t="s">
+      <c r="E3" s="15"/>
+      <c r="F3" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="12" t="s">
+      <c r="H3" s="12"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="12"/>
+      <c r="Q3" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="11" t="s">
+      <c r="R3" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="S3" s="11"/>
+      <c r="S3" s="12"/>
     </row>
     <row r="4" s="1" customFormat="1" ht="13" customHeight="1" spans="1:19">
       <c r="A4" s="7">
@@ -1704,31 +1534,31 @@
       <c r="D4" s="7">
         <v>1</v>
       </c>
-      <c r="E4" s="13"/>
-      <c r="F4" s="14" t="s">
+      <c r="E4" s="15"/>
+      <c r="F4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="12" t="s">
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="13"/>
+      <c r="M4" s="12"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+      <c r="P4" s="12"/>
+      <c r="Q4" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="R4" s="15" t="s">
+      <c r="R4" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="S4" s="11"/>
-    </row>
-    <row r="5" s="1" customFormat="1" ht="16.5" spans="1:19">
+      <c r="S4" s="12"/>
+    </row>
+    <row r="5" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A5" s="7">
         <v>4</v>
       </c>
@@ -1739,31 +1569,31 @@
       <c r="D5" s="7">
         <v>1</v>
       </c>
-      <c r="E5" s="13"/>
-      <c r="F5" s="16" t="s">
+      <c r="E5" s="15"/>
+      <c r="F5" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="12" t="s">
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12"/>
+      <c r="P5" s="12"/>
+      <c r="Q5" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="R5" s="15" t="s">
+      <c r="R5" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="S5" s="11"/>
-    </row>
-    <row r="6" s="1" customFormat="1" ht="16.5" spans="1:19">
+      <c r="S5" s="12"/>
+    </row>
+    <row r="6" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A6" s="7">
         <v>5</v>
       </c>
@@ -1774,813 +1604,910 @@
       <c r="D6" s="7">
         <v>1</v>
       </c>
-      <c r="E6" s="13"/>
-      <c r="F6" s="14" t="s">
+      <c r="E6" s="15"/>
+      <c r="F6" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="12" t="s">
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="13"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="12"/>
+      <c r="Q6" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="R6" s="15" t="s">
+      <c r="R6" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="S6" s="11"/>
-    </row>
-    <row r="7" s="1" customFormat="1" ht="16.5" spans="1:19">
+      <c r="S6" s="12"/>
+    </row>
+    <row r="7" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A7" s="7">
         <v>6</v>
       </c>
-      <c r="B7" s="11"/>
+      <c r="B7" s="12"/>
       <c r="C7" s="8">
         <v>17003440</v>
       </c>
       <c r="D7" s="7">
         <v>1</v>
       </c>
-      <c r="E7" s="13"/>
-      <c r="F7" s="14" t="s">
+      <c r="E7" s="15"/>
+      <c r="F7" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="12" t="s">
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="13"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="R7" s="15" t="s">
+      <c r="R7" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="S7" s="11"/>
-    </row>
-    <row r="8" s="1" customFormat="1" ht="16.5" spans="1:19">
+      <c r="S7" s="12"/>
+    </row>
+    <row r="8" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A8" s="7">
         <v>7</v>
       </c>
-      <c r="B8" s="11"/>
+      <c r="B8" s="12"/>
       <c r="C8" s="8">
         <v>17003110</v>
       </c>
-      <c r="D8" s="17">
+      <c r="D8" s="16">
         <v>1</v>
       </c>
-      <c r="E8" s="13"/>
-      <c r="F8" s="14" t="s">
+      <c r="E8" s="15"/>
+      <c r="F8" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="12" t="s">
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
+      <c r="Q8" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="R8" s="15" t="s">
+      <c r="R8" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="S8" s="11"/>
+      <c r="S8" s="12"/>
     </row>
     <row r="9" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A9" s="7">
         <v>8</v>
       </c>
-      <c r="B9" s="11"/>
+      <c r="B9" s="12"/>
       <c r="C9" s="8">
         <v>17000240</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="16">
         <v>1</v>
       </c>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11" t="s">
+      <c r="E9" s="12"/>
+      <c r="F9" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="12" t="s">
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="12"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="R9" s="15" t="s">
+      <c r="R9" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="S9" s="11"/>
-    </row>
-    <row r="10" s="1" customFormat="1" ht="16.5" spans="1:19">
+      <c r="S9" s="12"/>
+    </row>
+    <row r="10" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A10" s="7">
         <v>9</v>
       </c>
-      <c r="B10" s="11"/>
+      <c r="B10" s="12"/>
       <c r="C10" s="8">
         <v>17003320</v>
       </c>
-      <c r="D10" s="17">
+      <c r="D10" s="16">
         <v>1</v>
       </c>
-      <c r="E10" s="11"/>
-      <c r="F10" s="8" t="s">
+      <c r="E10" s="12"/>
+      <c r="F10" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="18" t="s">
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R10" s="19" t="s">
+      <c r="R10" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="S10" s="11"/>
-    </row>
-    <row r="11" s="1" customFormat="1" ht="16.5" spans="1:19">
+      <c r="S10" s="12"/>
+    </row>
+    <row r="11" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A11" s="7">
         <v>10</v>
       </c>
-      <c r="B11" s="11"/>
+      <c r="B11" s="12"/>
       <c r="C11" s="8">
         <v>17003330</v>
       </c>
       <c r="D11" s="7">
         <v>1</v>
       </c>
-      <c r="E11" s="11"/>
-      <c r="F11" s="8" t="s">
+      <c r="E11" s="12"/>
+      <c r="F11" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="18" t="s">
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="12"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R11" s="19" t="s">
+      <c r="R11" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S11" s="11"/>
-    </row>
-    <row r="12" s="1" customFormat="1" ht="16.5" spans="1:19">
+      <c r="S11" s="12"/>
+    </row>
+    <row r="12" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A12" s="7">
         <v>11</v>
       </c>
-      <c r="B12" s="11"/>
+      <c r="B12" s="12"/>
       <c r="C12" s="8">
         <v>17003100</v>
       </c>
       <c r="D12" s="7">
         <v>1</v>
       </c>
-      <c r="E12" s="11"/>
-      <c r="F12" s="8" t="s">
+      <c r="E12" s="12"/>
+      <c r="F12" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="18" t="s">
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="12"/>
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R12" s="19" t="s">
+      <c r="R12" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S12" s="11"/>
+      <c r="S12" s="12"/>
     </row>
     <row r="13" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A13" s="7">
         <v>12</v>
       </c>
-      <c r="B13" s="11"/>
+      <c r="B13" s="12"/>
       <c r="C13" s="8">
         <v>17003240</v>
       </c>
       <c r="D13" s="7">
         <v>1</v>
       </c>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11" t="s">
+      <c r="E13" s="12"/>
+      <c r="F13" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="18" t="s">
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="13"/>
+      <c r="M13" s="12"/>
+      <c r="N13" s="12"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R13" s="19" t="s">
+      <c r="R13" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S13" s="11"/>
+      <c r="S13" s="12"/>
     </row>
     <row r="14" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A14" s="7">
         <v>13</v>
       </c>
-      <c r="B14" s="11"/>
+      <c r="B14" s="12"/>
       <c r="C14" s="8">
         <v>72700220</v>
       </c>
       <c r="D14" s="7">
         <v>1</v>
       </c>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11" t="s">
+      <c r="E14" s="12"/>
+      <c r="F14" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="18" t="s">
+      <c r="H14" s="12"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="13"/>
+      <c r="M14" s="12"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="R14" s="19" t="s">
+      <c r="R14" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="S14" s="11"/>
+      <c r="S14" s="12"/>
     </row>
     <row r="15" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A15" s="7">
         <v>14</v>
       </c>
-      <c r="B15" s="11"/>
+      <c r="B15" s="12"/>
       <c r="C15" s="8">
         <v>74700690</v>
       </c>
       <c r="D15" s="7">
         <v>1</v>
       </c>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11" t="s">
+      <c r="E15" s="12"/>
+      <c r="F15" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="G15" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="18" t="s">
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="13"/>
+      <c r="M15" s="12"/>
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="R15" s="19" t="s">
+      <c r="R15" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="S15" s="11"/>
+      <c r="S15" s="12"/>
     </row>
     <row r="16" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A16" s="7">
         <v>15</v>
       </c>
-      <c r="B16" s="11"/>
+      <c r="B16" s="12"/>
       <c r="C16" s="8">
         <v>52900013</v>
       </c>
       <c r="D16" s="7">
         <v>1</v>
       </c>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11" t="s">
+      <c r="E16" s="12"/>
+      <c r="F16" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="G16" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="18" t="s">
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="12"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="13"/>
+      <c r="M16" s="12"/>
+      <c r="N16" s="12"/>
+      <c r="O16" s="12"/>
+      <c r="P16" s="12"/>
+      <c r="Q16" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="R16" s="19" t="s">
+      <c r="R16" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S16" s="11"/>
+      <c r="S16" s="12"/>
     </row>
     <row r="17" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A17" s="7">
         <v>16</v>
       </c>
-      <c r="B17" s="11"/>
+      <c r="B17" s="12"/>
       <c r="C17" s="8">
         <v>41000505</v>
       </c>
-      <c r="D17" s="17">
+      <c r="D17" s="16">
         <v>1</v>
       </c>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11" t="s">
+      <c r="E17" s="12"/>
+      <c r="F17" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="G17" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="18" t="s">
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="12"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="12"/>
+      <c r="Q17" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R17" s="19" t="s">
+      <c r="R17" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S17" s="11"/>
+      <c r="S17" s="12"/>
     </row>
     <row r="18" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A18" s="7">
         <v>17</v>
       </c>
-      <c r="B18" s="11"/>
+      <c r="B18" s="12"/>
       <c r="C18" s="8">
         <v>41000045</v>
       </c>
-      <c r="D18" s="17">
+      <c r="D18" s="16">
         <v>1</v>
       </c>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11" t="s">
+      <c r="E18" s="12"/>
+      <c r="F18" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="G18" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="G18" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="18" t="s">
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="12"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="12"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="12"/>
+      <c r="Q18" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R18" s="19" t="s">
+      <c r="R18" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S18" s="11"/>
+      <c r="S18" s="12"/>
     </row>
     <row r="19" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A19" s="7">
         <v>18</v>
       </c>
-      <c r="B19" s="11"/>
+      <c r="B19" s="12"/>
       <c r="C19" s="8">
         <v>91000908</v>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="16">
         <v>1</v>
       </c>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11" t="s">
+      <c r="E19" s="12"/>
+      <c r="F19" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="G19" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="G19" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="18" t="s">
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="12"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
+      <c r="P19" s="12"/>
+      <c r="Q19" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R19" s="19" t="s">
+      <c r="R19" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S19" s="11"/>
+      <c r="S19" s="12"/>
     </row>
     <row r="20" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A20" s="7">
         <v>19</v>
       </c>
-      <c r="B20" s="11"/>
+      <c r="B20" s="12"/>
       <c r="C20" s="8">
         <v>76700420</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="7">
         <v>1</v>
       </c>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11" t="s">
+      <c r="E20" s="12"/>
+      <c r="F20" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="G20" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="G20" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="18" t="s">
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="12"/>
+      <c r="Q20" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="R20" s="19" t="s">
+      <c r="R20" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S20" s="11"/>
+      <c r="S20" s="12"/>
     </row>
     <row r="21" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A21" s="7">
         <v>20</v>
       </c>
-      <c r="B21" s="11"/>
+      <c r="B21" s="12"/>
       <c r="C21" s="8">
         <v>60250009</v>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="7">
         <v>1</v>
       </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="11" t="s">
+      <c r="E21" s="12"/>
+      <c r="F21" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="G21" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="H21" s="11"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="18" t="s">
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="12"/>
+      <c r="Q21" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="R21" s="19" t="s">
+      <c r="R21" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S21" s="11"/>
+      <c r="S21" s="12"/>
     </row>
     <row r="22" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A22" s="7">
         <v>21</v>
       </c>
-      <c r="B22" s="11"/>
+      <c r="B22" s="12"/>
       <c r="C22" s="8">
         <v>41000501</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="16">
         <v>1</v>
       </c>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11" t="s">
-        <v>54</v>
-      </c>
-      <c r="G22" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="11"/>
-      <c r="P22" s="11"/>
-      <c r="Q22" s="18" t="s">
+      <c r="E22" s="12"/>
+      <c r="F22" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="G22" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="H22" s="12"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="12"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="12"/>
+      <c r="Q22" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R22" s="19" t="s">
+      <c r="R22" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S22" s="11"/>
+      <c r="S22" s="12"/>
     </row>
     <row r="23" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A23" s="7">
         <v>22</v>
       </c>
-      <c r="B23" s="11"/>
+      <c r="B23" s="12"/>
       <c r="C23" s="8">
         <v>52800100</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="16">
         <v>1</v>
       </c>
-      <c r="E23" s="11"/>
-      <c r="F23" s="13" t="s">
+      <c r="E23" s="12"/>
+      <c r="F23" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="G23" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="12"/>
+      <c r="Q23" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="H23" s="11"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="11"/>
-      <c r="K23" s="11"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="11"/>
-      <c r="P23" s="11"/>
-      <c r="Q23" s="18" t="s">
+      <c r="R23" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="R23" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="S23" s="11"/>
+      <c r="S23" s="12"/>
     </row>
     <row r="24" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A24" s="7">
         <v>23</v>
       </c>
-      <c r="B24" s="11"/>
+      <c r="B24" s="12"/>
       <c r="C24" s="8">
         <v>52800030</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="16">
         <v>1</v>
       </c>
-      <c r="E24" s="11"/>
-      <c r="F24" s="13" t="s">
+      <c r="E24" s="12"/>
+      <c r="F24" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="G24" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="G24" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="H24" s="11"/>
-      <c r="I24" s="11"/>
-      <c r="J24" s="11"/>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="18" t="s">
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="12"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="12"/>
+      <c r="Q24" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="R24" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="R24" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="S24" s="11"/>
+      <c r="S24" s="12"/>
     </row>
     <row r="25" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A25" s="7">
         <v>24</v>
       </c>
-      <c r="B25" s="11"/>
+      <c r="B25" s="12"/>
       <c r="C25" s="8">
         <v>91000939</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="16">
         <v>1</v>
       </c>
-      <c r="E25" s="11"/>
-      <c r="F25" s="13" t="s">
+      <c r="E25" s="12"/>
+      <c r="F25" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="G25" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="G25" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="H25" s="11"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="18" t="s">
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="12"/>
+      <c r="P25" s="12"/>
+      <c r="Q25" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R25" s="19" t="s">
+      <c r="R25" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="S25" s="11"/>
+      <c r="S25" s="12"/>
     </row>
     <row r="26" s="1" customFormat="1" ht="14.5" spans="1:19">
       <c r="A26" s="7">
         <v>25</v>
       </c>
-      <c r="B26" s="11"/>
+      <c r="B26" s="12"/>
       <c r="C26" s="8">
         <v>91000917</v>
       </c>
-      <c r="D26" s="20">
+      <c r="D26" s="16">
         <v>1</v>
       </c>
-      <c r="E26" s="11"/>
-      <c r="F26" s="11" t="s">
+      <c r="E26" s="12"/>
+      <c r="F26" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="G26" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="G26" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="H26" s="11"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="11"/>
-      <c r="K26" s="11"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11"/>
-      <c r="O26" s="11"/>
-      <c r="P26" s="11"/>
-      <c r="Q26" s="18" t="s">
+      <c r="H26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="12"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="13"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="12"/>
+      <c r="P26" s="12"/>
+      <c r="Q26" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="R26" s="19" t="s">
+      <c r="R26" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="S26" s="11"/>
+      <c r="S26" s="12"/>
     </row>
     <row r="27" spans="1:19">
       <c r="A27" s="24"/>
-      <c r="C27" s="25">
+      <c r="B27" s="25"/>
+      <c r="C27" s="26">
         <v>17000050</v>
       </c>
-      <c r="D27" s="26">
+      <c r="D27" s="27">
         <v>2</v>
       </c>
-      <c r="F27" t="s">
-        <v>75</v>
-      </c>
+      <c r="E27" s="25"/>
+      <c r="F27" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="25"/>
     </row>
     <row r="28" spans="1:19">
       <c r="A28" s="24"/>
+      <c r="B28" s="25"/>
+      <c r="C28" s="25"/>
+      <c r="D28" s="25"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="25"/>
+      <c r="K28" s="25"/>
     </row>
     <row r="29" spans="1:19">
       <c r="A29" s="24"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="25"/>
+      <c r="K29" s="25"/>
     </row>
     <row r="30" spans="1:19">
       <c r="A30" s="24"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="25"/>
+      <c r="K30" s="25"/>
     </row>
     <row r="31" spans="1:19">
       <c r="A31" s="24"/>
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="25"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="25"/>
+      <c r="J31" s="25"/>
+      <c r="K31" s="25"/>
     </row>
     <row r="32" spans="1:19">
       <c r="A32" s="24"/>
-    </row>
-    <row r="33" spans="1:1">
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="25"/>
+      <c r="J32" s="25"/>
+      <c r="K32" s="25"/>
+    </row>
+    <row r="33" spans="1:11">
       <c r="A33" s="24"/>
-    </row>
-    <row r="34" spans="1:1">
+      <c r="B33" s="25"/>
+      <c r="C33" s="25"/>
+      <c r="D33" s="25"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="25"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="25"/>
+      <c r="J33" s="25"/>
+      <c r="K33" s="25"/>
+    </row>
+    <row r="34" spans="1:11">
       <c r="A34" s="24"/>
-    </row>
-    <row r="35" spans="1:1">
+      <c r="B34" s="25"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="25"/>
+      <c r="J34" s="25"/>
+      <c r="K34" s="25"/>
+    </row>
+    <row r="35" spans="1:11">
       <c r="A35" s="24"/>
-    </row>
-    <row r="36" spans="1:1">
+      <c r="B35" s="25"/>
+      <c r="C35" s="25"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="25"/>
+      <c r="H35" s="25"/>
+      <c r="I35" s="25"/>
+      <c r="J35" s="25"/>
+      <c r="K35" s="25"/>
+    </row>
+    <row r="36" spans="1:11">
       <c r="A36" s="24"/>
-    </row>
-    <row r="37" spans="1:1">
-      <c r="A37" s="24"/>
-    </row>
-    <row r="38" spans="1:1">
-      <c r="A38" s="24"/>
-    </row>
-    <row r="39" spans="1:1">
-      <c r="A39" s="24"/>
-    </row>
-    <row r="40" spans="1:1">
-      <c r="A40" s="24"/>
-    </row>
-    <row r="41" spans="1:1">
-      <c r="A41" s="24"/>
-    </row>
-    <row r="42" spans="1:1">
-      <c r="A42" s="24"/>
-    </row>
-    <row r="43" spans="1:1">
-      <c r="A43" s="24"/>
-    </row>
-    <row r="44" spans="1:1">
-      <c r="A44" s="24"/>
-    </row>
-    <row r="45" spans="1:1">
-      <c r="A45" s="24"/>
-    </row>
-    <row r="46" spans="1:1">
-      <c r="A46" s="24"/>
-    </row>
-    <row r="47" spans="1:1">
-      <c r="A47" s="24"/>
-    </row>
-    <row r="48" spans="1:1">
-      <c r="A48" s="24"/>
+      <c r="B36" s="25"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="25"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="25"/>
+      <c r="G36" s="25"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="25"/>
+      <c r="J36" s="25"/>
+      <c r="K36" s="25"/>
+    </row>
+    <row r="37" spans="1:11">
+      <c r="A37" s="28"/>
+    </row>
+    <row r="38" spans="1:11">
+      <c r="A38" s="28"/>
+    </row>
+    <row r="39" spans="1:11">
+      <c r="A39" s="28"/>
+    </row>
+    <row r="40" spans="1:11">
+      <c r="A40" s="28"/>
+    </row>
+    <row r="41" spans="1:11">
+      <c r="A41" s="28"/>
+    </row>
+    <row r="42" spans="1:11">
+      <c r="A42" s="28"/>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="A43" s="28"/>
+    </row>
+    <row r="44" spans="1:11">
+      <c r="A44" s="28"/>
+    </row>
+    <row r="45" spans="1:11">
+      <c r="A45" s="28"/>
+    </row>
+    <row r="46" spans="1:11">
+      <c r="A46" s="28"/>
+    </row>
+    <row r="47" spans="1:11">
+      <c r="A47" s="28"/>
+    </row>
+    <row r="48" spans="1:11">
+      <c r="A48" s="28"/>
     </row>
     <row r="49" spans="1:1">
-      <c r="A49" s="24"/>
+      <c r="A49" s="28"/>
     </row>
     <row r="50" spans="1:1">
-      <c r="A50" s="24"/>
+      <c r="A50" s="28"/>
     </row>
     <row r="51" spans="1:1">
-      <c r="A51" s="24"/>
+      <c r="A51" s="28"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2">

</xml_diff>

<commit_message>
Refine app workflow and refresh generated workbook artifacts.
Simplify app logic and update template/info/output Excel files to match the latest packing list generation behavior.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/info.xlsx
+++ b/info.xlsx
@@ -1504,7 +1504,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1600,9 +1600,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment/>
@@ -3419,7 +3416,9 @@
         <v>4500468584</v>
       </c>
       <c r="H57" s="7"/>
-      <c r="I57" s="7"/>
+      <c r="I57" s="7">
+        <v>4</v>
+      </c>
     </row>
     <row r="58" spans="1:9">
       <c r="A58" s="8">
@@ -3444,7 +3443,9 @@
         <v>4500468584</v>
       </c>
       <c r="H58" s="7"/>
-      <c r="I58" s="7"/>
+      <c r="I58" s="7">
+        <v>7.8</v>
+      </c>
     </row>
     <row r="59" spans="1:9">
       <c r="A59" s="8">
@@ -3469,7 +3470,9 @@
         <v>4500468584</v>
       </c>
       <c r="H59" s="7"/>
-      <c r="I59" s="7"/>
+      <c r="I59" s="7">
+        <v>21</v>
+      </c>
     </row>
     <row r="60" spans="1:9">
       <c r="A60" s="8">
@@ -3494,7 +3497,9 @@
         <v>4500468584</v>
       </c>
       <c r="H60" s="7"/>
-      <c r="I60" s="7"/>
+      <c r="I60" s="7">
+        <v>21</v>
+      </c>
     </row>
     <row r="61" spans="1:9">
       <c r="A61" s="8">
@@ -3546,7 +3551,9 @@
         <v>4500468584</v>
       </c>
       <c r="H62" s="7"/>
-      <c r="I62" s="7"/>
+      <c r="I62" s="7">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="63" spans="1:9">
       <c r="A63" s="8">
@@ -3596,7 +3603,9 @@
         <v>4500468584</v>
       </c>
       <c r="H64" s="7"/>
-      <c r="I64" s="7"/>
+      <c r="I64" s="7">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="65" spans="1:9">
       <c r="A65" s="8">
@@ -3621,7 +3630,9 @@
         <v>4500468584</v>
       </c>
       <c r="H65" s="7"/>
-      <c r="I65" s="7"/>
+      <c r="I65" s="7">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="66" spans="1:9">
       <c r="A66" s="8">
@@ -3646,7 +3657,9 @@
         <v>4500468584</v>
       </c>
       <c r="H66" s="7"/>
-      <c r="I66" s="7"/>
+      <c r="I66" s="7">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="67" spans="1:9">
       <c r="A67" s="8">
@@ -3671,7 +3684,9 @@
         <v>4500468584</v>
       </c>
       <c r="H67" s="7"/>
-      <c r="I67" s="7"/>
+      <c r="I67" s="7">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="68" spans="1:9">
       <c r="A68" s="8">
@@ -3696,7 +3711,9 @@
         <v>4500468584</v>
       </c>
       <c r="H68" s="7"/>
-      <c r="I68" s="7"/>
+      <c r="I68" s="7">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="69" spans="1:9">
       <c r="A69" s="8">
@@ -3721,7 +3738,9 @@
         <v>4500468584</v>
       </c>
       <c r="H69" s="7"/>
-      <c r="I69" s="7"/>
+      <c r="I69" s="7">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="70" spans="1:9">
       <c r="A70" s="8">
@@ -6242,17 +6261,17 @@
       <c r="A166" s="8">
         <v>165</v>
       </c>
-      <c r="B166" s="34">
+      <c r="B166" s="7">
         <v>86070423</v>
       </c>
-      <c r="C166" s="34" t="s">
+      <c r="C166" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="D166" s="34"/>
-      <c r="E166" s="34">
-        <v>1</v>
-      </c>
-      <c r="F166" s="34"/>
+      <c r="D166" s="7"/>
+      <c r="E166" s="7">
+        <v>1</v>
+      </c>
+      <c r="F166" s="7"/>
       <c r="G166" s="33">
         <v>4500468584</v>
       </c>
@@ -6263,17 +6282,17 @@
       <c r="A167" s="8">
         <v>166</v>
       </c>
-      <c r="B167" s="34">
+      <c r="B167" s="7">
         <v>42011002</v>
       </c>
-      <c r="C167" s="34" t="s">
+      <c r="C167" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="D167" s="34"/>
-      <c r="E167" s="34">
-        <v>3</v>
-      </c>
-      <c r="F167" s="34"/>
+      <c r="D167" s="7"/>
+      <c r="E167" s="7">
+        <v>3</v>
+      </c>
+      <c r="F167" s="7"/>
       <c r="G167" s="33">
         <v>4500468584</v>
       </c>
@@ -6284,19 +6303,19 @@
       <c r="A168" s="8">
         <v>167</v>
       </c>
-      <c r="B168" s="34">
+      <c r="B168" s="7">
         <v>52000040</v>
       </c>
-      <c r="C168" s="34" t="s">
+      <c r="C168" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="D168" s="34">
+      <c r="D168" s="7">
         <v>5702</v>
       </c>
-      <c r="E168" s="34">
+      <c r="E168" s="7">
         <v>2</v>
       </c>
-      <c r="F168" s="34"/>
+      <c r="F168" s="7"/>
       <c r="G168" s="33">
         <v>4500468584</v>
       </c>
@@ -6307,17 +6326,17 @@
       <c r="A169" s="8">
         <v>168</v>
       </c>
-      <c r="B169" s="34">
+      <c r="B169" s="7">
         <v>52001020</v>
       </c>
-      <c r="C169" s="34" t="s">
+      <c r="C169" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="D169" s="34"/>
-      <c r="E169" s="34">
-        <v>1</v>
-      </c>
-      <c r="F169" s="34"/>
+      <c r="D169" s="7"/>
+      <c r="E169" s="7">
+        <v>1</v>
+      </c>
+      <c r="F169" s="7"/>
       <c r="G169" s="33">
         <v>4500468584</v>
       </c>
@@ -6328,19 +6347,19 @@
       <c r="A170" s="8">
         <v>169</v>
       </c>
-      <c r="B170" s="34">
+      <c r="B170" s="7">
         <v>17003440</v>
       </c>
-      <c r="C170" s="34" t="s">
+      <c r="C170" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="D170" s="34">
+      <c r="D170" s="7">
         <v>6402</v>
       </c>
-      <c r="E170" s="34">
+      <c r="E170" s="7">
         <v>11</v>
       </c>
-      <c r="F170" s="34"/>
+      <c r="F170" s="7"/>
       <c r="G170" s="33">
         <v>4500468584</v>
       </c>
@@ -6351,19 +6370,19 @@
       <c r="A171" s="8">
         <v>170</v>
       </c>
-      <c r="B171" s="34">
+      <c r="B171" s="7">
         <v>52001000</v>
       </c>
-      <c r="C171" s="34" t="s">
+      <c r="C171" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="D171" s="34">
+      <c r="D171" s="7">
         <v>6401</v>
       </c>
-      <c r="E171" s="34">
-        <v>1</v>
-      </c>
-      <c r="F171" s="34"/>
+      <c r="E171" s="7">
+        <v>1</v>
+      </c>
+      <c r="F171" s="7"/>
       <c r="G171" s="33">
         <v>4500468584</v>
       </c>
@@ -6374,17 +6393,17 @@
       <c r="A172" s="8">
         <v>171</v>
       </c>
-      <c r="B172" s="34">
+      <c r="B172" s="7">
         <v>17004250</v>
       </c>
-      <c r="C172" s="34" t="s">
+      <c r="C172" s="7" t="s">
         <v>201</v>
       </c>
-      <c r="D172" s="34"/>
-      <c r="E172" s="34">
+      <c r="D172" s="7"/>
+      <c r="E172" s="7">
         <v>11</v>
       </c>
-      <c r="F172" s="34"/>
+      <c r="F172" s="7"/>
       <c r="G172" s="33">
         <v>4500468584</v>
       </c>
@@ -6395,22 +6414,22 @@
       <c r="A173" s="8">
         <v>172</v>
       </c>
-      <c r="B173" s="34">
+      <c r="B173" s="7">
         <v>86070436</v>
       </c>
-      <c r="C173" s="34" t="s">
+      <c r="C173" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="D173" s="34">
+      <c r="D173" s="7">
         <v>5901</v>
       </c>
-      <c r="E173" s="34">
-        <v>3</v>
-      </c>
-      <c r="F173" s="34" t="s">
+      <c r="E173" s="7">
+        <v>3</v>
+      </c>
+      <c r="F173" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="G173" s="34">
+      <c r="G173" s="7">
         <v>4500468584</v>
       </c>
       <c r="H173" s="7"/>
@@ -6420,22 +6439,22 @@
       <c r="A174" s="8">
         <v>173</v>
       </c>
-      <c r="B174" s="34">
+      <c r="B174" s="7">
         <v>86070437</v>
       </c>
-      <c r="C174" s="34" t="s">
+      <c r="C174" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="D174" s="34">
+      <c r="D174" s="7">
         <v>5701</v>
       </c>
-      <c r="E174" s="34">
+      <c r="E174" s="7">
         <v>2</v>
       </c>
-      <c r="F174" s="34" t="s">
+      <c r="F174" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="G174" s="34">
+      <c r="G174" s="7">
         <v>4500468584</v>
       </c>
       <c r="H174" s="7"/>
@@ -6445,22 +6464,22 @@
       <c r="A175" s="8">
         <v>174</v>
       </c>
-      <c r="B175" s="34">
+      <c r="B175" s="7">
         <v>86070437</v>
       </c>
-      <c r="C175" s="34" t="s">
+      <c r="C175" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="D175" s="34">
+      <c r="D175" s="7">
         <v>5702</v>
       </c>
-      <c r="E175" s="34">
-        <v>1</v>
-      </c>
-      <c r="F175" s="34" t="s">
+      <c r="E175" s="7">
+        <v>1</v>
+      </c>
+      <c r="F175" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="G175" s="34">
+      <c r="G175" s="7">
         <v>4500468584</v>
       </c>
       <c r="H175" s="7"/>
@@ -6470,22 +6489,22 @@
       <c r="A176" s="8">
         <v>175</v>
       </c>
-      <c r="B176" s="34">
+      <c r="B176" s="7">
         <v>86070438</v>
       </c>
-      <c r="C176" s="34" t="s">
+      <c r="C176" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="D176" s="34">
+      <c r="D176" s="7">
         <v>5702</v>
       </c>
-      <c r="E176" s="34">
-        <v>3</v>
-      </c>
-      <c r="F176" s="34" t="s">
+      <c r="E176" s="7">
+        <v>3</v>
+      </c>
+      <c r="F176" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="G176" s="34">
+      <c r="G176" s="7">
         <v>4500468584</v>
       </c>
       <c r="H176" s="7"/>
@@ -6495,22 +6514,22 @@
       <c r="A177" s="8">
         <v>176</v>
       </c>
-      <c r="B177" s="34">
+      <c r="B177" s="7">
         <v>86070439</v>
       </c>
-      <c r="C177" s="34" t="s">
+      <c r="C177" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="D177" s="34">
+      <c r="D177" s="7">
         <v>5701</v>
       </c>
-      <c r="E177" s="34">
+      <c r="E177" s="7">
         <v>2</v>
       </c>
-      <c r="F177" s="34" t="s">
+      <c r="F177" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="G177" s="34">
+      <c r="G177" s="7">
         <v>4500468584</v>
       </c>
       <c r="H177" s="7"/>
@@ -6520,22 +6539,22 @@
       <c r="A178" s="8">
         <v>177</v>
       </c>
-      <c r="B178" s="34">
+      <c r="B178" s="7">
         <v>86070439</v>
       </c>
-      <c r="C178" s="34" t="s">
+      <c r="C178" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="D178" s="34">
+      <c r="D178" s="7">
         <v>6301</v>
       </c>
-      <c r="E178" s="34">
-        <v>1</v>
-      </c>
-      <c r="F178" s="34" t="s">
+      <c r="E178" s="7">
+        <v>1</v>
+      </c>
+      <c r="F178" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="G178" s="34">
+      <c r="G178" s="7">
         <v>4500468584</v>
       </c>
       <c r="H178" s="7"/>
@@ -6545,20 +6564,20 @@
       <c r="A179" s="8">
         <v>178</v>
       </c>
-      <c r="B179" s="34">
+      <c r="B179" s="7">
         <v>52800039</v>
       </c>
-      <c r="C179" s="34" t="s">
+      <c r="C179" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="D179" s="34">
+      <c r="D179" s="7">
         <v>6302</v>
       </c>
-      <c r="E179" s="34">
+      <c r="E179" s="7">
         <v>2</v>
       </c>
-      <c r="F179" s="34"/>
-      <c r="G179" s="34">
+      <c r="F179" s="7"/>
+      <c r="G179" s="7">
         <v>4500468584</v>
       </c>
       <c r="H179" s="7"/>
@@ -6568,20 +6587,20 @@
       <c r="A180" s="8">
         <v>179</v>
       </c>
-      <c r="B180" s="35">
+      <c r="B180" s="34">
         <v>85070008</v>
       </c>
-      <c r="C180" s="35" t="s">
+      <c r="C180" s="34" t="s">
         <v>207</v>
       </c>
-      <c r="D180" s="35">
+      <c r="D180" s="34">
         <v>6401</v>
       </c>
-      <c r="E180" s="35">
+      <c r="E180" s="34">
         <v>5</v>
       </c>
-      <c r="F180" s="34"/>
-      <c r="G180" s="34">
+      <c r="F180" s="7"/>
+      <c r="G180" s="7">
         <v>4500468584</v>
       </c>
       <c r="H180" s="7"/>
@@ -6591,20 +6610,20 @@
       <c r="A181" s="8">
         <v>180</v>
       </c>
-      <c r="B181" s="35">
+      <c r="B181" s="34">
         <v>85070010</v>
       </c>
-      <c r="C181" s="35" t="s">
+      <c r="C181" s="34" t="s">
         <v>208</v>
       </c>
-      <c r="D181" s="35">
+      <c r="D181" s="34">
         <v>6402</v>
       </c>
-      <c r="E181" s="35">
-        <v>3</v>
-      </c>
-      <c r="F181" s="34"/>
-      <c r="G181" s="34">
+      <c r="E181" s="34">
+        <v>3</v>
+      </c>
+      <c r="F181" s="7"/>
+      <c r="G181" s="7">
         <v>4500468584</v>
       </c>
       <c r="H181" s="7"/>
@@ -6614,20 +6633,20 @@
       <c r="A182" s="8">
         <v>181</v>
       </c>
-      <c r="B182" s="36">
+      <c r="B182" s="35">
         <v>85070017</v>
       </c>
-      <c r="C182" s="35" t="s">
+      <c r="C182" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="D182" s="35">
+      <c r="D182" s="34">
         <v>6402</v>
       </c>
-      <c r="E182" s="35">
+      <c r="E182" s="34">
         <v>8</v>
       </c>
-      <c r="F182" s="34"/>
-      <c r="G182" s="34">
+      <c r="F182" s="7"/>
+      <c r="G182" s="7">
         <v>4500468584</v>
       </c>
       <c r="H182" s="7"/>
@@ -6637,20 +6656,20 @@
       <c r="A183" s="8">
         <v>182</v>
       </c>
-      <c r="B183" s="36">
+      <c r="B183" s="35">
         <v>85070017</v>
       </c>
-      <c r="C183" s="35" t="s">
+      <c r="C183" s="34" t="s">
         <v>209</v>
       </c>
-      <c r="D183" s="35">
+      <c r="D183" s="34">
         <v>6402</v>
       </c>
-      <c r="E183" s="35">
-        <v>1</v>
-      </c>
-      <c r="F183" s="34"/>
-      <c r="G183" s="34">
+      <c r="E183" s="34">
+        <v>1</v>
+      </c>
+      <c r="F183" s="7"/>
+      <c r="G183" s="7">
         <v>4500468584</v>
       </c>
       <c r="H183" s="7"/>
@@ -6660,20 +6679,20 @@
       <c r="A184" s="8">
         <v>183</v>
       </c>
-      <c r="B184" s="35">
+      <c r="B184" s="34">
         <v>85070037</v>
       </c>
-      <c r="C184" s="35" t="s">
+      <c r="C184" s="34" t="s">
         <v>210</v>
       </c>
-      <c r="D184" s="35">
+      <c r="D184" s="34">
         <v>6402</v>
       </c>
-      <c r="E184" s="35">
-        <v>1</v>
-      </c>
-      <c r="F184" s="34"/>
-      <c r="G184" s="34">
+      <c r="E184" s="34">
+        <v>1</v>
+      </c>
+      <c r="F184" s="7"/>
+      <c r="G184" s="7">
         <v>4500468584</v>
       </c>
       <c r="H184" s="7"/>
@@ -6683,20 +6702,20 @@
       <c r="A185" s="8">
         <v>184</v>
       </c>
-      <c r="B185" s="35">
+      <c r="B185" s="34">
         <v>85070042</v>
       </c>
-      <c r="C185" s="35" t="s">
+      <c r="C185" s="34" t="s">
         <v>211</v>
       </c>
-      <c r="D185" s="35">
+      <c r="D185" s="34">
         <v>6402</v>
       </c>
-      <c r="E185" s="35">
-        <v>3</v>
-      </c>
-      <c r="F185" s="34"/>
-      <c r="G185" s="34">
+      <c r="E185" s="34">
+        <v>3</v>
+      </c>
+      <c r="F185" s="7"/>
+      <c r="G185" s="7">
         <v>4500468584</v>
       </c>
       <c r="H185" s="7"/>
@@ -6706,20 +6725,20 @@
       <c r="A186" s="8">
         <v>185</v>
       </c>
-      <c r="B186" s="35">
+      <c r="B186" s="34">
         <v>86070210</v>
       </c>
-      <c r="C186" s="35" t="s">
+      <c r="C186" s="34" t="s">
         <v>212</v>
       </c>
-      <c r="D186" s="35">
+      <c r="D186" s="34">
         <v>6402</v>
       </c>
-      <c r="E186" s="35">
-        <v>1</v>
-      </c>
-      <c r="F186" s="34"/>
-      <c r="G186" s="34">
+      <c r="E186" s="34">
+        <v>1</v>
+      </c>
+      <c r="F186" s="7"/>
+      <c r="G186" s="7">
         <v>4500468584</v>
       </c>
       <c r="H186" s="7"/>
@@ -6729,20 +6748,20 @@
       <c r="A187" s="8">
         <v>186</v>
       </c>
-      <c r="B187" s="35">
+      <c r="B187" s="34">
         <v>86070385</v>
       </c>
-      <c r="C187" s="35" t="s">
+      <c r="C187" s="34" t="s">
         <v>213</v>
       </c>
-      <c r="D187" s="35">
+      <c r="D187" s="34">
         <v>6402</v>
       </c>
-      <c r="E187" s="35">
-        <v>1</v>
-      </c>
-      <c r="F187" s="34"/>
-      <c r="G187" s="34">
+      <c r="E187" s="34">
+        <v>1</v>
+      </c>
+      <c r="F187" s="7"/>
+      <c r="G187" s="7">
         <v>4500468584</v>
       </c>
       <c r="H187" s="7"/>
@@ -6752,20 +6771,20 @@
       <c r="A188" s="8">
         <v>187</v>
       </c>
-      <c r="B188" s="35">
+      <c r="B188" s="34">
         <v>86070386</v>
       </c>
-      <c r="C188" s="35" t="s">
+      <c r="C188" s="34" t="s">
         <v>214</v>
       </c>
-      <c r="D188" s="35">
+      <c r="D188" s="34">
         <v>6402</v>
       </c>
-      <c r="E188" s="35">
-        <v>1</v>
-      </c>
-      <c r="F188" s="34"/>
-      <c r="G188" s="34">
+      <c r="E188" s="34">
+        <v>1</v>
+      </c>
+      <c r="F188" s="7"/>
+      <c r="G188" s="7">
         <v>4500468584</v>
       </c>
       <c r="H188" s="7"/>
@@ -6775,20 +6794,20 @@
       <c r="A189" s="8">
         <v>188</v>
       </c>
-      <c r="B189" s="35">
+      <c r="B189" s="34">
         <v>86070387</v>
       </c>
-      <c r="C189" s="35" t="s">
+      <c r="C189" s="34" t="s">
         <v>215</v>
       </c>
-      <c r="D189" s="35">
+      <c r="D189" s="34">
         <v>6402</v>
       </c>
-      <c r="E189" s="35">
-        <v>1</v>
-      </c>
-      <c r="F189" s="34"/>
-      <c r="G189" s="34">
+      <c r="E189" s="34">
+        <v>1</v>
+      </c>
+      <c r="F189" s="7"/>
+      <c r="G189" s="7">
         <v>4500468584</v>
       </c>
       <c r="H189" s="7"/>
@@ -6798,20 +6817,20 @@
       <c r="A190" s="8">
         <v>189</v>
       </c>
-      <c r="B190" s="35">
+      <c r="B190" s="34">
         <v>86070388</v>
       </c>
-      <c r="C190" s="35" t="s">
+      <c r="C190" s="34" t="s">
         <v>216</v>
       </c>
-      <c r="D190" s="35">
+      <c r="D190" s="34">
         <v>6402</v>
       </c>
-      <c r="E190" s="35">
-        <v>1</v>
-      </c>
-      <c r="F190" s="34"/>
-      <c r="G190" s="34">
+      <c r="E190" s="34">
+        <v>1</v>
+      </c>
+      <c r="F190" s="7"/>
+      <c r="G190" s="7">
         <v>4500468584</v>
       </c>
       <c r="H190" s="7"/>
@@ -6821,20 +6840,20 @@
       <c r="A191" s="8">
         <v>190</v>
       </c>
-      <c r="B191" s="35">
+      <c r="B191" s="34">
         <v>86070390</v>
       </c>
-      <c r="C191" s="35" t="s">
+      <c r="C191" s="34" t="s">
         <v>217</v>
       </c>
-      <c r="D191" s="35">
+      <c r="D191" s="34">
         <v>6402</v>
       </c>
-      <c r="E191" s="35">
-        <v>3</v>
-      </c>
-      <c r="F191" s="34"/>
-      <c r="G191" s="34">
+      <c r="E191" s="34">
+        <v>3</v>
+      </c>
+      <c r="F191" s="7"/>
+      <c r="G191" s="7">
         <v>4500468584</v>
       </c>
       <c r="H191" s="7"/>
@@ -6844,20 +6863,20 @@
       <c r="A192" s="8">
         <v>191</v>
       </c>
-      <c r="B192" s="35">
+      <c r="B192" s="34">
         <v>86070391</v>
       </c>
-      <c r="C192" s="35" t="s">
+      <c r="C192" s="34" t="s">
         <v>218</v>
       </c>
-      <c r="D192" s="35">
+      <c r="D192" s="34">
         <v>6402</v>
       </c>
-      <c r="E192" s="35">
-        <v>1</v>
-      </c>
-      <c r="F192" s="34"/>
-      <c r="G192" s="34">
+      <c r="E192" s="34">
+        <v>1</v>
+      </c>
+      <c r="F192" s="7"/>
+      <c r="G192" s="7">
         <v>4500468584</v>
       </c>
       <c r="H192" s="7"/>
@@ -6867,20 +6886,20 @@
       <c r="A193" s="8">
         <v>192</v>
       </c>
-      <c r="B193" s="35">
+      <c r="B193" s="34">
         <v>86070392</v>
       </c>
-      <c r="C193" s="35" t="s">
+      <c r="C193" s="34" t="s">
         <v>219</v>
       </c>
-      <c r="D193" s="35">
+      <c r="D193" s="34">
         <v>6402</v>
       </c>
-      <c r="E193" s="35">
-        <v>3</v>
-      </c>
-      <c r="F193" s="34"/>
-      <c r="G193" s="34">
+      <c r="E193" s="34">
+        <v>3</v>
+      </c>
+      <c r="F193" s="7"/>
+      <c r="G193" s="7">
         <v>4500468584</v>
       </c>
       <c r="H193" s="7"/>
@@ -6890,20 +6909,20 @@
       <c r="A194" s="8">
         <v>193</v>
       </c>
-      <c r="B194" s="35">
+      <c r="B194" s="34">
         <v>86070397</v>
       </c>
-      <c r="C194" s="35" t="s">
+      <c r="C194" s="34" t="s">
         <v>220</v>
       </c>
-      <c r="D194" s="35">
+      <c r="D194" s="34">
         <v>6402</v>
       </c>
-      <c r="E194" s="35">
-        <v>3</v>
-      </c>
-      <c r="F194" s="34"/>
-      <c r="G194" s="34">
+      <c r="E194" s="34">
+        <v>3</v>
+      </c>
+      <c r="F194" s="7"/>
+      <c r="G194" s="7">
         <v>4500468584</v>
       </c>
       <c r="H194" s="7"/>
@@ -6913,20 +6932,20 @@
       <c r="A195" s="8">
         <v>194</v>
       </c>
-      <c r="B195" s="35">
+      <c r="B195" s="34">
         <v>86070398</v>
       </c>
-      <c r="C195" s="35" t="s">
+      <c r="C195" s="34" t="s">
         <v>221</v>
       </c>
-      <c r="D195" s="35">
+      <c r="D195" s="34">
         <v>6402</v>
       </c>
-      <c r="E195" s="35">
-        <v>3</v>
-      </c>
-      <c r="F195" s="34"/>
-      <c r="G195" s="34">
+      <c r="E195" s="34">
+        <v>3</v>
+      </c>
+      <c r="F195" s="7"/>
+      <c r="G195" s="7">
         <v>4500468584</v>
       </c>
       <c r="H195" s="7"/>
@@ -6936,20 +6955,20 @@
       <c r="A196" s="8">
         <v>195</v>
       </c>
-      <c r="B196" s="35">
+      <c r="B196" s="34">
         <v>86070399</v>
       </c>
-      <c r="C196" s="35" t="s">
+      <c r="C196" s="34" t="s">
         <v>222</v>
       </c>
-      <c r="D196" s="35">
+      <c r="D196" s="34">
         <v>6402</v>
       </c>
-      <c r="E196" s="35">
-        <v>3</v>
-      </c>
-      <c r="F196" s="34"/>
-      <c r="G196" s="34">
+      <c r="E196" s="34">
+        <v>3</v>
+      </c>
+      <c r="F196" s="7"/>
+      <c r="G196" s="7">
         <v>4500468584</v>
       </c>
       <c r="H196" s="7"/>
@@ -6959,20 +6978,20 @@
       <c r="A197" s="8">
         <v>196</v>
       </c>
-      <c r="B197" s="35">
+      <c r="B197" s="34">
         <v>86070406</v>
       </c>
-      <c r="C197" s="35" t="s">
+      <c r="C197" s="34" t="s">
         <v>223</v>
       </c>
-      <c r="D197" s="35">
+      <c r="D197" s="34">
         <v>6402</v>
       </c>
-      <c r="E197" s="35">
-        <v>1</v>
-      </c>
-      <c r="F197" s="34"/>
-      <c r="G197" s="34">
+      <c r="E197" s="34">
+        <v>1</v>
+      </c>
+      <c r="F197" s="7"/>
+      <c r="G197" s="7">
         <v>4500468584</v>
       </c>
       <c r="H197" s="7"/>
@@ -6982,20 +7001,20 @@
       <c r="A198" s="8">
         <v>197</v>
       </c>
-      <c r="B198" s="35">
+      <c r="B198" s="34">
         <v>86070407</v>
       </c>
-      <c r="C198" s="35" t="s">
+      <c r="C198" s="34" t="s">
         <v>224</v>
       </c>
-      <c r="D198" s="35">
+      <c r="D198" s="34">
         <v>6402</v>
       </c>
-      <c r="E198" s="35">
-        <v>3</v>
-      </c>
-      <c r="F198" s="34"/>
-      <c r="G198" s="34">
+      <c r="E198" s="34">
+        <v>3</v>
+      </c>
+      <c r="F198" s="7"/>
+      <c r="G198" s="7">
         <v>4500468584</v>
       </c>
       <c r="H198" s="7"/>
@@ -7005,20 +7024,20 @@
       <c r="A199" s="8">
         <v>198</v>
       </c>
-      <c r="B199" s="35">
+      <c r="B199" s="34">
         <v>86070408</v>
       </c>
-      <c r="C199" s="35" t="s">
+      <c r="C199" s="34" t="s">
         <v>225</v>
       </c>
-      <c r="D199" s="35">
+      <c r="D199" s="34">
         <v>6402</v>
       </c>
-      <c r="E199" s="35">
-        <v>3</v>
-      </c>
-      <c r="F199" s="34"/>
-      <c r="G199" s="34">
+      <c r="E199" s="34">
+        <v>3</v>
+      </c>
+      <c r="F199" s="7"/>
+      <c r="G199" s="7">
         <v>4500468584</v>
       </c>
       <c r="H199" s="7"/>
@@ -7028,20 +7047,20 @@
       <c r="A200" s="8">
         <v>199</v>
       </c>
-      <c r="B200" s="35">
+      <c r="B200" s="34">
         <v>86070411</v>
       </c>
-      <c r="C200" s="35" t="s">
+      <c r="C200" s="34" t="s">
         <v>226</v>
       </c>
-      <c r="D200" s="35">
+      <c r="D200" s="34">
         <v>6402</v>
       </c>
-      <c r="E200" s="35">
+      <c r="E200" s="34">
         <v>2</v>
       </c>
-      <c r="F200" s="34"/>
-      <c r="G200" s="34">
+      <c r="F200" s="7"/>
+      <c r="G200" s="7">
         <v>4500468584</v>
       </c>
       <c r="H200" s="7"/>
@@ -7051,20 +7070,20 @@
       <c r="A201" s="8">
         <v>200</v>
       </c>
-      <c r="B201" s="35">
+      <c r="B201" s="34">
         <v>86070422</v>
       </c>
-      <c r="C201" s="35" t="s">
+      <c r="C201" s="34" t="s">
         <v>227</v>
       </c>
-      <c r="D201" s="35">
+      <c r="D201" s="34">
         <v>6402</v>
       </c>
-      <c r="E201" s="35">
-        <v>1</v>
-      </c>
-      <c r="F201" s="34"/>
-      <c r="G201" s="34">
+      <c r="E201" s="34">
+        <v>1</v>
+      </c>
+      <c r="F201" s="7"/>
+      <c r="G201" s="7">
         <v>4500468584</v>
       </c>
       <c r="H201" s="7"/>
@@ -7074,20 +7093,20 @@
       <c r="A202" s="8">
         <v>201</v>
       </c>
-      <c r="B202" s="35">
+      <c r="B202" s="34">
         <v>86070423</v>
       </c>
-      <c r="C202" s="35" t="s">
+      <c r="C202" s="34" t="s">
         <v>228</v>
       </c>
-      <c r="D202" s="35">
+      <c r="D202" s="34">
         <v>6402</v>
       </c>
-      <c r="E202" s="35">
-        <v>1</v>
-      </c>
-      <c r="F202" s="34"/>
-      <c r="G202" s="34">
+      <c r="E202" s="34">
+        <v>1</v>
+      </c>
+      <c r="F202" s="7"/>
+      <c r="G202" s="7">
         <v>4500468584</v>
       </c>
       <c r="H202" s="7"/>
@@ -7097,20 +7116,20 @@
       <c r="A203" s="8">
         <v>202</v>
       </c>
-      <c r="B203" s="35">
+      <c r="B203" s="34">
         <v>86070424</v>
       </c>
-      <c r="C203" s="35" t="s">
+      <c r="C203" s="34" t="s">
         <v>229</v>
       </c>
-      <c r="D203" s="35">
+      <c r="D203" s="34">
         <v>6402</v>
       </c>
-      <c r="E203" s="35">
+      <c r="E203" s="34">
         <v>2</v>
       </c>
-      <c r="F203" s="34"/>
-      <c r="G203" s="34">
+      <c r="F203" s="7"/>
+      <c r="G203" s="7">
         <v>4500468584</v>
       </c>
       <c r="H203" s="7"/>
@@ -7120,20 +7139,20 @@
       <c r="A204" s="8">
         <v>203</v>
       </c>
-      <c r="B204" s="35">
+      <c r="B204" s="34">
         <v>86070425</v>
       </c>
-      <c r="C204" s="35" t="s">
+      <c r="C204" s="34" t="s">
         <v>230</v>
       </c>
-      <c r="D204" s="35">
+      <c r="D204" s="34">
         <v>6402</v>
       </c>
-      <c r="E204" s="35">
-        <v>3</v>
-      </c>
-      <c r="F204" s="34"/>
-      <c r="G204" s="34">
+      <c r="E204" s="34">
+        <v>3</v>
+      </c>
+      <c r="F204" s="7"/>
+      <c r="G204" s="7">
         <v>4500468584</v>
       </c>
       <c r="H204" s="7"/>
@@ -7143,20 +7162,20 @@
       <c r="A205" s="8">
         <v>204</v>
       </c>
-      <c r="B205" s="35">
+      <c r="B205" s="34">
         <v>86070426</v>
       </c>
-      <c r="C205" s="35" t="s">
+      <c r="C205" s="34" t="s">
         <v>231</v>
       </c>
-      <c r="D205" s="35">
+      <c r="D205" s="34">
         <v>6402</v>
       </c>
-      <c r="E205" s="35">
-        <v>3</v>
-      </c>
-      <c r="F205" s="34"/>
-      <c r="G205" s="34">
+      <c r="E205" s="34">
+        <v>3</v>
+      </c>
+      <c r="F205" s="7"/>
+      <c r="G205" s="7">
         <v>4500468584</v>
       </c>
       <c r="H205" s="7"/>
@@ -7166,20 +7185,20 @@
       <c r="A206" s="8">
         <v>205</v>
       </c>
-      <c r="B206" s="35">
+      <c r="B206" s="34">
         <v>86070430</v>
       </c>
-      <c r="C206" s="35" t="s">
+      <c r="C206" s="34" t="s">
         <v>232</v>
       </c>
-      <c r="D206" s="35">
+      <c r="D206" s="34">
         <v>6402</v>
       </c>
-      <c r="E206" s="35">
+      <c r="E206" s="34">
         <v>2</v>
       </c>
-      <c r="F206" s="34"/>
-      <c r="G206" s="34">
+      <c r="F206" s="7"/>
+      <c r="G206" s="7">
         <v>4500468584</v>
       </c>
       <c r="H206" s="7"/>
@@ -7189,20 +7208,20 @@
       <c r="A207" s="8">
         <v>206</v>
       </c>
-      <c r="B207" s="35">
+      <c r="B207" s="34">
         <v>86070431</v>
       </c>
-      <c r="C207" s="35" t="s">
+      <c r="C207" s="34" t="s">
         <v>233</v>
       </c>
-      <c r="D207" s="35">
+      <c r="D207" s="34">
         <v>6402</v>
       </c>
-      <c r="E207" s="35">
-        <v>3</v>
-      </c>
-      <c r="F207" s="34"/>
-      <c r="G207" s="34">
+      <c r="E207" s="34">
+        <v>3</v>
+      </c>
+      <c r="F207" s="7"/>
+      <c r="G207" s="7">
         <v>4500468584</v>
       </c>
       <c r="H207" s="7"/>
@@ -7212,20 +7231,20 @@
       <c r="A208" s="8">
         <v>207</v>
       </c>
-      <c r="B208" s="35">
+      <c r="B208" s="34">
         <v>86070432</v>
       </c>
-      <c r="C208" s="35" t="s">
+      <c r="C208" s="34" t="s">
         <v>234</v>
       </c>
-      <c r="D208" s="35">
+      <c r="D208" s="34">
         <v>6402</v>
       </c>
-      <c r="E208" s="35">
-        <v>3</v>
-      </c>
-      <c r="F208" s="34"/>
-      <c r="G208" s="34">
+      <c r="E208" s="34">
+        <v>3</v>
+      </c>
+      <c r="F208" s="7"/>
+      <c r="G208" s="7">
         <v>4500468584</v>
       </c>
       <c r="H208" s="7"/>
@@ -7235,20 +7254,20 @@
       <c r="A209" s="8">
         <v>208</v>
       </c>
-      <c r="B209" s="35">
+      <c r="B209" s="34">
         <v>86070433</v>
       </c>
-      <c r="C209" s="35" t="s">
+      <c r="C209" s="34" t="s">
         <v>235</v>
       </c>
-      <c r="D209" s="35">
+      <c r="D209" s="34">
         <v>6402</v>
       </c>
-      <c r="E209" s="35">
-        <v>3</v>
-      </c>
-      <c r="F209" s="34"/>
-      <c r="G209" s="34">
+      <c r="E209" s="34">
+        <v>3</v>
+      </c>
+      <c r="F209" s="7"/>
+      <c r="G209" s="7">
         <v>4500468584</v>
       </c>
       <c r="H209" s="7"/>

</xml_diff>